<commit_message>
text type fixes to make model run
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
+++ b/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kjh_local\NEXTgroup_local\2025_local\2. EPS\업데이트 파일\eps-southkorea-3.3.1_2025update_v4.0.3\InputData\bldgs\SYDEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\bldgs\SYDEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C5CF29-75C1-4297-BED8-6C3C181082EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3AC53B6-CDCC-4172-BF4D-E3E350C26836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="670" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="435" yWindow="4005" windowWidth="18405" windowHeight="10920" tabRatio="670" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="23" r:id="rId1"/>
@@ -581,7 +581,7 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <rFont val="맑은 고딕"/>
+        <rFont val="Calibri"/>
         <family val="3"/>
         <charset val="129"/>
         <scheme val="minor"/>
@@ -591,7 +591,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <rFont val="맑은 고딕"/>
+        <rFont val="Calibri"/>
         <family val="3"/>
         <charset val="129"/>
         <scheme val="minor"/>
@@ -979,20 +979,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="0.00_ "/>
-    <numFmt numFmtId="177" formatCode="#,##0.00_ "/>
-    <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="179" formatCode="#,##0_);[Red]\(#,##0\)"/>
-    <numFmt numFmtId="182" formatCode="0_);[Red]\(0\)"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="0.00_ "/>
+    <numFmt numFmtId="167" formatCode="#,##0.00_ "/>
+    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="35">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1000,7 +998,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1027,7 +1025,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1035,20 +1033,20 @@
       <b/>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1057,7 +1055,7 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1065,28 +1063,28 @@
     <font>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1094,7 +1092,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1108,7 +1106,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1117,7 +1115,7 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1125,7 +1123,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1133,7 +1131,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1141,7 +1139,7 @@
     <font>
       <b/>
       <sz val="14"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1150,7 +1148,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1159,7 +1157,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1168,14 +1166,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1196,7 +1194,7 @@
       <b/>
       <sz val="14"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1205,7 +1203,7 @@
       <u/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1214,7 +1212,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1" tint="4.9989318521683403E-2"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1222,7 +1220,7 @@
     <font>
       <sz val="11"/>
       <color theme="1" tint="4.9989318521683403E-2"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1230,14 +1228,14 @@
     <font>
       <sz val="10"/>
       <color theme="1" tint="4.9989318521683403E-2"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1253,7 +1251,7 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -2245,7 +2243,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
@@ -2256,7 +2254,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="290">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2279,10 +2277,10 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2312,13 +2310,13 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="9" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="19" fillId="0" borderId="6" xfId="9" applyFont="1" applyBorder="1">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="6" xfId="9" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="18" fillId="0" borderId="6" xfId="9" applyFont="1" applyBorder="1">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="6" xfId="9" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2365,7 +2363,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2375,7 +2373,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="11"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2383,7 +2381,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2395,8 +2393,8 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="176" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2411,7 +2409,7 @@
     <xf numFmtId="0" fontId="10" fillId="14" borderId="66" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="65" xfId="10" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="10" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2443,43 +2441,43 @@
     <xf numFmtId="0" fontId="30" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="11" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="11" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2488,34 +2486,34 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="11" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="11" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="29" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="29" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2527,7 +2525,7 @@
     <xf numFmtId="0" fontId="29" fillId="5" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2539,67 +2537,67 @@
     <xf numFmtId="0" fontId="30" fillId="5" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="56" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="56" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="53" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="53" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="58" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="58" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="56" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="56" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="53" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="53" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="38" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="58" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="58" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="12" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="12" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2614,182 +2612,182 @@
     <xf numFmtId="0" fontId="30" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="68" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="68" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="71" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="71" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="73" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="73" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="53" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="11" applyFont="1"/>
-    <xf numFmtId="179" fontId="29" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="29" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="10" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="10" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="0" borderId="9" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="0" borderId="9" xfId="9" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="8" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="8" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="7" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="7" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="38" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2798,13 +2796,13 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="76" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="76" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2816,16 +2814,16 @@
     <xf numFmtId="0" fontId="30" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2834,22 +2832,22 @@
     <xf numFmtId="0" fontId="30" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="8" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -2882,67 +2880,67 @@
     <xf numFmtId="0" fontId="30" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="30" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2954,28 +2952,28 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2984,7 +2982,7 @@
     <xf numFmtId="0" fontId="30" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3000,29 +2998,32 @@
     <xf numFmtId="4" fontId="24" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3031,13 +3032,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="12" borderId="65" xfId="10" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -3062,22 +3060,21 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Comma [0]" xfId="9" builtinId="6"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Footnotes: top row" xfId="6" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Header: bottom row" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Header: top rows" xfId="8" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Parent row" xfId="4" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Table title" xfId="3" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="쉼표 [0]" xfId="9" builtinId="6"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="10" xr:uid="{DE05B990-2924-4931-9EDF-3EEC26F286F8}"/>
     <cellStyle name="표준 4" xfId="12" xr:uid="{DAAD85BD-8C63-49E9-B5C2-89FAD72545EE}"/>
-    <cellStyle name="하이퍼링크" xfId="11" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3419,12 +3416,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84495FF6-49F8-4752-902B-BDC955084312}">
   <dimension ref="A1:F77"/>
-  <sheetFormatPr defaultRowHeight="17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.08203125" customWidth="1"/>
+    <col min="1" max="1" width="17.109375" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3517,12 +3514,12 @@
         <v>160</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="17.5" thickBot="1">
+    <row r="21" spans="1:2" ht="15" thickBot="1">
       <c r="A21" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="17.5" thickBot="1">
+    <row r="22" spans="1:2" ht="15" thickBot="1">
       <c r="A22" s="60">
         <v>2023</v>
       </c>
@@ -3611,19 +3608,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2951CA25-AEBA-4E14-BF02-109840382943}">
   <dimension ref="A1:AE702"/>
-  <sheetFormatPr defaultRowHeight="17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="6.58203125" customWidth="1"/>
-    <col min="2" max="2" width="11.58203125" customWidth="1"/>
-    <col min="3" max="3" width="4.08203125" customWidth="1"/>
-    <col min="4" max="4" width="26.58203125" customWidth="1"/>
-    <col min="5" max="22" width="11.58203125" customWidth="1"/>
-    <col min="23" max="23" width="4.08203125" customWidth="1"/>
-    <col min="24" max="24" width="26.58203125" customWidth="1"/>
-    <col min="25" max="26" width="11.58203125" customWidth="1"/>
+    <col min="1" max="1" width="6.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="3" max="3" width="4.109375" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" customWidth="1"/>
+    <col min="5" max="22" width="11.5546875" customWidth="1"/>
+    <col min="23" max="23" width="4.109375" customWidth="1"/>
+    <col min="24" max="24" width="26.5546875" customWidth="1"/>
+    <col min="25" max="26" width="11.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:24" s="6" customFormat="1" ht="25.5">
+    <row r="1" spans="3:24" s="6" customFormat="1" ht="21">
       <c r="C1" s="263" t="s">
         <v>130</v>
       </c>
@@ -3668,10 +3665,10 @@
       <c r="X4" s="25"/>
     </row>
     <row r="5" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C5" s="269" t="s">
+      <c r="C5" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="269"/>
+      <c r="D5" s="267"/>
       <c r="E5" s="72" t="s">
         <v>79</v>
       </c>
@@ -3726,14 +3723,14 @@
       <c r="V5" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W5" s="273" t="s">
+      <c r="W5" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X5" s="269"/>
+      <c r="X5" s="267"/>
     </row>
     <row r="6" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C6" s="270"/>
-      <c r="D6" s="270"/>
+      <c r="C6" s="268"/>
+      <c r="D6" s="268"/>
       <c r="E6" s="75" t="s">
         <v>22</v>
       </c>
@@ -3788,8 +3785,8 @@
       <c r="V6" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W6" s="274"/>
-      <c r="X6" s="270"/>
+      <c r="W6" s="270"/>
+      <c r="X6" s="268"/>
     </row>
     <row r="7" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C7" s="78" t="s">
@@ -5349,7 +5346,7 @@
       <c r="W34" s="93"/>
       <c r="X34" s="93"/>
     </row>
-    <row r="37" spans="3:31" s="6" customFormat="1" ht="21">
+    <row r="37" spans="3:31" s="6" customFormat="1" ht="18">
       <c r="C37" s="19" t="s">
         <v>117</v>
       </c>
@@ -5378,10 +5375,10 @@
       <c r="X38" s="29"/>
     </row>
     <row r="39" spans="3:31" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C39" s="269" t="s">
+      <c r="C39" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D39" s="269"/>
+      <c r="D39" s="267"/>
       <c r="E39" s="104" t="s">
         <v>79</v>
       </c>
@@ -5436,10 +5433,10 @@
       <c r="V39" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W39" s="269" t="s">
+      <c r="W39" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="X39" s="269"/>
+      <c r="X39" s="267"/>
       <c r="AA39"/>
       <c r="AB39"/>
       <c r="AC39"/>
@@ -5447,8 +5444,8 @@
       <c r="AE39"/>
     </row>
     <row r="40" spans="3:31" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C40" s="270"/>
-      <c r="D40" s="270"/>
+      <c r="C40" s="268"/>
+      <c r="D40" s="268"/>
       <c r="E40" s="108" t="s">
         <v>22</v>
       </c>
@@ -5503,8 +5500,8 @@
       <c r="V40" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W40" s="270"/>
-      <c r="X40" s="270"/>
+      <c r="W40" s="268"/>
+      <c r="X40" s="268"/>
     </row>
     <row r="41" spans="3:31" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C41" s="78" t="s">
@@ -7384,7 +7381,7 @@
       <c r="W73" s="93"/>
       <c r="X73" s="93"/>
     </row>
-    <row r="76" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="76" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C76" s="19" t="s">
         <v>116</v>
       </c>
@@ -7416,10 +7413,10 @@
       <c r="X77" s="29"/>
     </row>
     <row r="78" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C78" s="269" t="s">
+      <c r="C78" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D78" s="269"/>
+      <c r="D78" s="267"/>
       <c r="E78" s="72" t="s">
         <v>79</v>
       </c>
@@ -7474,14 +7471,14 @@
       <c r="V78" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W78" s="273" t="s">
+      <c r="W78" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X78" s="269"/>
+      <c r="X78" s="267"/>
     </row>
     <row r="79" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C79" s="270"/>
-      <c r="D79" s="270"/>
+      <c r="C79" s="268"/>
+      <c r="D79" s="268"/>
       <c r="E79" s="75" t="s">
         <v>22</v>
       </c>
@@ -7536,8 +7533,8 @@
       <c r="V79" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W79" s="274"/>
-      <c r="X79" s="270"/>
+      <c r="W79" s="270"/>
+      <c r="X79" s="268"/>
     </row>
     <row r="80" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C80" s="78" t="s">
@@ -9417,7 +9414,7 @@
       <c r="W112" s="103"/>
       <c r="X112" s="103"/>
     </row>
-    <row r="115" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="115" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C115" s="19" t="s">
         <v>115</v>
       </c>
@@ -9425,7 +9422,7 @@
       <c r="E115" s="10"/>
       <c r="F115" s="10"/>
     </row>
-    <row r="116" spans="3:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="116" spans="3:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="C116" s="16"/>
       <c r="D116" s="16"/>
       <c r="E116" s="16"/>
@@ -9448,10 +9445,10 @@
       <c r="X116" s="29"/>
     </row>
     <row r="117" spans="3:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="C117" s="269" t="s">
+      <c r="C117" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D117" s="269"/>
+      <c r="D117" s="267"/>
       <c r="E117" s="72" t="s">
         <v>79</v>
       </c>
@@ -9506,14 +9503,14 @@
       <c r="V117" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W117" s="273" t="s">
+      <c r="W117" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X117" s="269"/>
+      <c r="X117" s="267"/>
     </row>
     <row r="118" spans="3:24" s="6" customFormat="1" ht="49.5" customHeight="1">
-      <c r="C118" s="270"/>
-      <c r="D118" s="270"/>
+      <c r="C118" s="268"/>
+      <c r="D118" s="268"/>
       <c r="E118" s="75" t="s">
         <v>22</v>
       </c>
@@ -9568,8 +9565,8 @@
       <c r="V118" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W118" s="274"/>
-      <c r="X118" s="270"/>
+      <c r="W118" s="270"/>
+      <c r="X118" s="268"/>
     </row>
     <row r="119" spans="3:24" s="12" customFormat="1">
       <c r="C119" s="78" t="s">
@@ -11337,7 +11334,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="149" spans="3:24" s="12" customFormat="1" ht="17.5" thickBot="1">
+    <row r="149" spans="3:24" s="12" customFormat="1" ht="15" thickBot="1">
       <c r="C149" s="96"/>
       <c r="D149" s="96" t="s">
         <v>24</v>
@@ -11425,7 +11422,7 @@
       <c r="W150" s="84"/>
       <c r="X150" s="84"/>
     </row>
-    <row r="151" spans="3:24" s="7" customFormat="1" ht="16">
+    <row r="151" spans="3:24" s="7" customFormat="1" ht="13.8">
       <c r="C151" s="103" t="s">
         <v>223</v>
       </c>
@@ -11451,7 +11448,7 @@
       <c r="W151" s="103"/>
       <c r="X151" s="103"/>
     </row>
-    <row r="154" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="154" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C154" s="19" t="s">
         <v>114</v>
       </c>
@@ -11480,10 +11477,10 @@
       <c r="X155" s="29"/>
     </row>
     <row r="156" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C156" s="269" t="s">
+      <c r="C156" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D156" s="269"/>
+      <c r="D156" s="267"/>
       <c r="E156" s="72" t="s">
         <v>79</v>
       </c>
@@ -11538,14 +11535,14 @@
       <c r="V156" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W156" s="273" t="s">
+      <c r="W156" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X156" s="269"/>
+      <c r="X156" s="267"/>
     </row>
     <row r="157" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C157" s="270"/>
-      <c r="D157" s="270"/>
+      <c r="C157" s="268"/>
+      <c r="D157" s="268"/>
       <c r="E157" s="75" t="s">
         <v>22</v>
       </c>
@@ -11600,8 +11597,8 @@
       <c r="V157" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W157" s="274"/>
-      <c r="X157" s="270"/>
+      <c r="W157" s="270"/>
+      <c r="X157" s="268"/>
     </row>
     <row r="158" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C158" s="78" t="s">
@@ -13481,7 +13478,7 @@
       <c r="W190" s="103"/>
       <c r="X190" s="103"/>
     </row>
-    <row r="193" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="193" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C193" s="19" t="s">
         <v>113</v>
       </c>
@@ -13512,10 +13509,10 @@
       <c r="X194" s="25"/>
     </row>
     <row r="195" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C195" s="269" t="s">
+      <c r="C195" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D195" s="269"/>
+      <c r="D195" s="267"/>
       <c r="E195" s="180" t="s">
         <v>79</v>
       </c>
@@ -13570,14 +13567,14 @@
       <c r="V195" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W195" s="273" t="s">
+      <c r="W195" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X195" s="269"/>
+      <c r="X195" s="267"/>
     </row>
     <row r="196" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C196" s="270"/>
-      <c r="D196" s="270"/>
+      <c r="C196" s="268"/>
+      <c r="D196" s="268"/>
       <c r="E196" s="181" t="s">
         <v>22</v>
       </c>
@@ -13632,8 +13629,8 @@
       <c r="V196" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W196" s="274"/>
-      <c r="X196" s="270"/>
+      <c r="W196" s="270"/>
+      <c r="X196" s="268"/>
     </row>
     <row r="197" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C197" s="78" t="s">
@@ -15155,7 +15152,7 @@
       <c r="W224" s="103"/>
       <c r="X224" s="103"/>
     </row>
-    <row r="227" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="227" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C227" s="19" t="s">
         <v>112</v>
       </c>
@@ -15186,10 +15183,10 @@
       <c r="X228" s="25"/>
     </row>
     <row r="229" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C229" s="269" t="s">
+      <c r="C229" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D229" s="269"/>
+      <c r="D229" s="267"/>
       <c r="E229" s="72" t="s">
         <v>79</v>
       </c>
@@ -15244,14 +15241,14 @@
       <c r="V229" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W229" s="273" t="s">
+      <c r="W229" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X229" s="269"/>
+      <c r="X229" s="267"/>
     </row>
     <row r="230" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C230" s="270"/>
-      <c r="D230" s="270"/>
+      <c r="C230" s="268"/>
+      <c r="D230" s="268"/>
       <c r="E230" s="75" t="s">
         <v>22</v>
       </c>
@@ -15306,8 +15303,8 @@
       <c r="V230" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W230" s="274"/>
-      <c r="X230" s="270"/>
+      <c r="W230" s="270"/>
+      <c r="X230" s="268"/>
     </row>
     <row r="231" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C231" s="78" t="s">
@@ -16829,14 +16826,14 @@
       <c r="W258" s="93"/>
       <c r="X258" s="93"/>
     </row>
-    <row r="261" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="261" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A261" s="19" t="s">
         <v>104</v>
       </c>
       <c r="B261" s="26"/>
       <c r="C261" s="12"/>
     </row>
-    <row r="262" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="262" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A262" s="16"/>
       <c r="B262" s="16"/>
       <c r="C262" s="17"/>
@@ -16861,11 +16858,11 @@
       <c r="X262" s="29"/>
     </row>
     <row r="263" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A263" s="269" t="s">
+      <c r="A263" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B263" s="269"/>
-      <c r="C263" s="269"/>
+      <c r="B263" s="267"/>
+      <c r="C263" s="267"/>
       <c r="D263" s="72" t="s">
         <v>79</v>
       </c>
@@ -16920,16 +16917,16 @@
       <c r="U263" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V263" s="273" t="s">
+      <c r="V263" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W263" s="269"/>
-      <c r="X263" s="269"/>
+      <c r="W263" s="267"/>
+      <c r="X263" s="267"/>
     </row>
     <row r="264" spans="1:24" s="6" customFormat="1">
-      <c r="A264" s="270"/>
-      <c r="B264" s="270"/>
-      <c r="C264" s="270"/>
+      <c r="A264" s="268"/>
+      <c r="B264" s="268"/>
+      <c r="C264" s="268"/>
       <c r="D264" s="75" t="s">
         <v>22</v>
       </c>
@@ -16984,9 +16981,9 @@
       <c r="U264" s="203" t="s">
         <v>44</v>
       </c>
-      <c r="V264" s="274"/>
-      <c r="W264" s="270"/>
-      <c r="X264" s="270"/>
+      <c r="V264" s="270"/>
+      <c r="W264" s="268"/>
+      <c r="X264" s="268"/>
     </row>
     <row r="265" spans="1:24" s="12" customFormat="1">
       <c r="A265" s="204" t="s">
@@ -17702,7 +17699,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="278" spans="1:24" s="12" customFormat="1" ht="17.5" thickBot="1">
+    <row r="278" spans="1:24" s="12" customFormat="1" ht="15" thickBot="1">
       <c r="A278" s="96"/>
       <c r="B278" s="96"/>
       <c r="C278" s="219" t="s">
@@ -17794,7 +17791,7 @@
       <c r="W279" s="220"/>
       <c r="X279" s="220"/>
     </row>
-    <row r="280" spans="1:24" s="7" customFormat="1" ht="16">
+    <row r="280" spans="1:24" s="7" customFormat="1" ht="13.8">
       <c r="A280" s="103" t="s">
         <v>231</v>
       </c>
@@ -17822,7 +17819,7 @@
       <c r="W280" s="103"/>
       <c r="X280" s="103"/>
     </row>
-    <row r="281" spans="1:24" s="7" customFormat="1" ht="16">
+    <row r="281" spans="1:24" s="7" customFormat="1" ht="13.8">
       <c r="A281" s="103" t="s">
         <v>84</v>
       </c>
@@ -17850,7 +17847,7 @@
       <c r="W281" s="103"/>
       <c r="X281" s="103"/>
     </row>
-    <row r="284" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="284" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A284" s="19" t="s">
         <v>103</v>
       </c>
@@ -17858,7 +17855,7 @@
       <c r="C284" s="12"/>
       <c r="X284" s="12"/>
     </row>
-    <row r="285" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="285" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A285" s="16"/>
       <c r="B285" s="16"/>
       <c r="C285" s="17"/>
@@ -17885,11 +17882,11 @@
       <c r="X285" s="27"/>
     </row>
     <row r="286" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A286" s="269" t="s">
+      <c r="A286" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B286" s="269"/>
-      <c r="C286" s="269"/>
+      <c r="B286" s="267"/>
+      <c r="C286" s="267"/>
       <c r="D286" s="221" t="s">
         <v>79</v>
       </c>
@@ -17944,16 +17941,16 @@
       <c r="U286" s="223" t="s">
         <v>62</v>
       </c>
-      <c r="V286" s="273" t="s">
+      <c r="V286" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W286" s="269"/>
-      <c r="X286" s="269"/>
+      <c r="W286" s="267"/>
+      <c r="X286" s="267"/>
     </row>
     <row r="287" spans="1:24" s="6" customFormat="1">
-      <c r="A287" s="270"/>
-      <c r="B287" s="270"/>
-      <c r="C287" s="270"/>
+      <c r="A287" s="268"/>
+      <c r="B287" s="268"/>
+      <c r="C287" s="268"/>
       <c r="D287" s="224" t="s">
         <v>22</v>
       </c>
@@ -18008,9 +18005,9 @@
       <c r="U287" s="226" t="s">
         <v>44</v>
       </c>
-      <c r="V287" s="274"/>
-      <c r="W287" s="270"/>
-      <c r="X287" s="270"/>
+      <c r="V287" s="270"/>
+      <c r="W287" s="268"/>
+      <c r="X287" s="268"/>
     </row>
     <row r="288" spans="1:24" s="12" customFormat="1">
       <c r="A288" s="78" t="s">
@@ -18726,7 +18723,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="301" spans="1:24" s="20" customFormat="1" ht="17.5" thickBot="1">
+    <row r="301" spans="1:24" s="20" customFormat="1" ht="15" thickBot="1">
       <c r="A301" s="96"/>
       <c r="B301" s="96"/>
       <c r="C301" s="233" t="s">
@@ -18874,12 +18871,12 @@
       <c r="W304" s="93"/>
       <c r="X304" s="93"/>
     </row>
-    <row r="307" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="307" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A307" s="19" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="308" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="308" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A308" s="16"/>
       <c r="B308" s="16"/>
       <c r="C308" s="16"/>
@@ -18906,11 +18903,11 @@
       <c r="X308" s="25"/>
     </row>
     <row r="309" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A309" s="269" t="s">
+      <c r="A309" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B309" s="269"/>
-      <c r="C309" s="269"/>
+      <c r="B309" s="267"/>
+      <c r="C309" s="267"/>
       <c r="D309" s="72" t="s">
         <v>79</v>
       </c>
@@ -18965,16 +18962,16 @@
       <c r="U309" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V309" s="273" t="s">
+      <c r="V309" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W309" s="269"/>
-      <c r="X309" s="269"/>
+      <c r="W309" s="267"/>
+      <c r="X309" s="267"/>
     </row>
     <row r="310" spans="1:24" s="6" customFormat="1">
-      <c r="A310" s="270"/>
-      <c r="B310" s="270"/>
-      <c r="C310" s="270"/>
+      <c r="A310" s="268"/>
+      <c r="B310" s="268"/>
+      <c r="C310" s="268"/>
       <c r="D310" s="75" t="s">
         <v>22</v>
       </c>
@@ -19029,16 +19026,16 @@
       <c r="U310" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V310" s="274"/>
-      <c r="W310" s="270"/>
-      <c r="X310" s="270"/>
+      <c r="V310" s="270"/>
+      <c r="W310" s="268"/>
+      <c r="X310" s="268"/>
     </row>
     <row r="311" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A311" s="277" t="s">
+      <c r="A311" s="273" t="s">
         <v>211</v>
       </c>
-      <c r="B311" s="277"/>
-      <c r="C311" s="278"/>
+      <c r="B311" s="273"/>
+      <c r="C311" s="274"/>
       <c r="D311" s="80">
         <v>692374.42799999856</v>
       </c>
@@ -19093,18 +19090,18 @@
       <c r="U311" s="83">
         <v>16879.359874472899</v>
       </c>
-      <c r="V311" s="277" t="s">
+      <c r="V311" s="273" t="s">
         <v>211</v>
       </c>
-      <c r="W311" s="277"/>
-      <c r="X311" s="278"/>
+      <c r="W311" s="273"/>
+      <c r="X311" s="274"/>
     </row>
     <row r="312" spans="1:24" s="9" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A312" s="271" t="s">
+      <c r="A312" s="272" t="s">
         <v>235</v>
       </c>
-      <c r="B312" s="271"/>
-      <c r="C312" s="272"/>
+      <c r="B312" s="272"/>
+      <c r="C312" s="275"/>
       <c r="D312" s="97">
         <v>1277579.9999999986</v>
       </c>
@@ -19159,11 +19156,11 @@
       <c r="U312" s="100">
         <v>31146.0558280888</v>
       </c>
-      <c r="V312" s="271" t="s">
+      <c r="V312" s="272" t="s">
         <v>235</v>
       </c>
-      <c r="W312" s="271"/>
-      <c r="X312" s="272"/>
+      <c r="W312" s="272"/>
+      <c r="X312" s="275"/>
     </row>
     <row r="313" spans="1:24" s="6" customFormat="1">
       <c r="A313" s="235"/>
@@ -19247,7 +19244,7 @@
       <c r="W315" s="93"/>
       <c r="X315" s="93"/>
     </row>
-    <row r="318" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="318" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A318" s="19" t="s">
         <v>101</v>
       </c>
@@ -19255,7 +19252,7 @@
       <c r="C318" s="12"/>
       <c r="X318" s="12"/>
     </row>
-    <row r="319" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="319" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A319" s="16"/>
       <c r="B319" s="16"/>
       <c r="C319" s="17"/>
@@ -19284,11 +19281,11 @@
       </c>
     </row>
     <row r="320" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A320" s="269" t="s">
+      <c r="A320" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B320" s="269"/>
-      <c r="C320" s="269"/>
+      <c r="B320" s="267"/>
+      <c r="C320" s="267"/>
       <c r="D320" s="72" t="s">
         <v>79</v>
       </c>
@@ -19343,16 +19340,16 @@
       <c r="U320" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V320" s="273" t="s">
+      <c r="V320" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W320" s="269"/>
-      <c r="X320" s="269"/>
+      <c r="W320" s="267"/>
+      <c r="X320" s="267"/>
     </row>
     <row r="321" spans="1:24" s="6" customFormat="1">
-      <c r="A321" s="270"/>
-      <c r="B321" s="270"/>
-      <c r="C321" s="270"/>
+      <c r="A321" s="268"/>
+      <c r="B321" s="268"/>
+      <c r="C321" s="268"/>
       <c r="D321" s="75" t="s">
         <v>22</v>
       </c>
@@ -19407,9 +19404,9 @@
       <c r="U321" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V321" s="274"/>
-      <c r="W321" s="270"/>
-      <c r="X321" s="270"/>
+      <c r="V321" s="270"/>
+      <c r="W321" s="268"/>
+      <c r="X321" s="268"/>
     </row>
     <row r="322" spans="1:24" s="12" customFormat="1">
       <c r="A322" s="78" t="s">
@@ -20125,7 +20122,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="335" spans="1:24" s="12" customFormat="1" ht="17.5" thickBot="1">
+    <row r="335" spans="1:24" s="12" customFormat="1" ht="15" thickBot="1">
       <c r="A335" s="84"/>
       <c r="B335" s="84"/>
       <c r="C335" s="233" t="s">
@@ -20301,7 +20298,7 @@
       <c r="W339" s="93"/>
       <c r="X339" s="93"/>
     </row>
-    <row r="342" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="342" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A342" s="19" t="s">
         <v>99</v>
       </c>
@@ -20333,11 +20330,11 @@
       <c r="X343" s="25"/>
     </row>
     <row r="344" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A344" s="269" t="s">
+      <c r="A344" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B344" s="269"/>
-      <c r="C344" s="269"/>
+      <c r="B344" s="267"/>
+      <c r="C344" s="267"/>
       <c r="D344" s="72" t="s">
         <v>79</v>
       </c>
@@ -20392,16 +20389,16 @@
       <c r="U344" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V344" s="273" t="s">
+      <c r="V344" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W344" s="269"/>
-      <c r="X344" s="275"/>
+      <c r="W344" s="267"/>
+      <c r="X344" s="276"/>
     </row>
     <row r="345" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A345" s="270"/>
-      <c r="B345" s="270"/>
-      <c r="C345" s="270"/>
+      <c r="A345" s="268"/>
+      <c r="B345" s="268"/>
+      <c r="C345" s="268"/>
       <c r="D345" s="75" t="s">
         <v>22</v>
       </c>
@@ -20456,16 +20453,16 @@
       <c r="U345" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V345" s="274"/>
-      <c r="W345" s="270"/>
-      <c r="X345" s="276"/>
+      <c r="V345" s="270"/>
+      <c r="W345" s="268"/>
+      <c r="X345" s="277"/>
     </row>
     <row r="346" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A346" s="277" t="s">
+      <c r="A346" s="273" t="s">
         <v>211</v>
       </c>
-      <c r="B346" s="277"/>
-      <c r="C346" s="278"/>
+      <c r="B346" s="273"/>
+      <c r="C346" s="274"/>
       <c r="D346" s="80">
         <v>3866.2734599999926</v>
       </c>
@@ -20527,11 +20524,11 @@
       <c r="X346" s="79"/>
     </row>
     <row r="347" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A347" s="271" t="s">
+      <c r="A347" s="272" t="s">
         <v>242</v>
       </c>
-      <c r="B347" s="271"/>
-      <c r="C347" s="272"/>
+      <c r="B347" s="272"/>
+      <c r="C347" s="275"/>
       <c r="D347" s="97">
         <v>9205.4129999999859</v>
       </c>
@@ -20586,11 +20583,11 @@
       <c r="U347" s="100">
         <v>173.15829496975101</v>
       </c>
-      <c r="V347" s="279" t="s">
+      <c r="V347" s="271" t="s">
         <v>242</v>
       </c>
-      <c r="W347" s="271"/>
-      <c r="X347" s="271"/>
+      <c r="W347" s="272"/>
+      <c r="X347" s="272"/>
     </row>
     <row r="348" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
       <c r="A348" s="220"/>
@@ -20702,7 +20699,7 @@
       <c r="W351" s="93"/>
       <c r="X351" s="93"/>
     </row>
-    <row r="353" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="353" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A353" s="19" t="s">
         <v>98</v>
       </c>
@@ -20710,7 +20707,7 @@
       <c r="C353" s="12"/>
       <c r="X353" s="12"/>
     </row>
-    <row r="354" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="354" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A354" s="16"/>
       <c r="B354" s="16"/>
       <c r="C354" s="17"/>
@@ -20737,11 +20734,11 @@
       <c r="X354" s="27"/>
     </row>
     <row r="355" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A355" s="269" t="s">
+      <c r="A355" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B355" s="269"/>
-      <c r="C355" s="269"/>
+      <c r="B355" s="267"/>
+      <c r="C355" s="267"/>
       <c r="D355" s="72" t="s">
         <v>79</v>
       </c>
@@ -20796,16 +20793,16 @@
       <c r="U355" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V355" s="273" t="s">
+      <c r="V355" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W355" s="269"/>
-      <c r="X355" s="275"/>
+      <c r="W355" s="267"/>
+      <c r="X355" s="276"/>
     </row>
     <row r="356" spans="1:24" s="6" customFormat="1">
-      <c r="A356" s="270"/>
-      <c r="B356" s="270"/>
-      <c r="C356" s="270"/>
+      <c r="A356" s="268"/>
+      <c r="B356" s="268"/>
+      <c r="C356" s="268"/>
       <c r="D356" s="75" t="s">
         <v>22</v>
       </c>
@@ -20860,16 +20857,16 @@
       <c r="U356" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V356" s="274"/>
-      <c r="W356" s="270"/>
-      <c r="X356" s="276"/>
+      <c r="V356" s="270"/>
+      <c r="W356" s="268"/>
+      <c r="X356" s="277"/>
     </row>
     <row r="357" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A357" s="277" t="s">
+      <c r="A357" s="273" t="s">
         <v>211</v>
       </c>
-      <c r="B357" s="277"/>
-      <c r="C357" s="278"/>
+      <c r="B357" s="273"/>
+      <c r="C357" s="274"/>
       <c r="D357" s="160">
         <v>209524.83999999997</v>
       </c>
@@ -20924,18 +20921,18 @@
       <c r="U357" s="164">
         <v>801.36</v>
       </c>
-      <c r="V357" s="277" t="s">
+      <c r="V357" s="273" t="s">
         <v>211</v>
       </c>
-      <c r="W357" s="277"/>
-      <c r="X357" s="278"/>
+      <c r="W357" s="273"/>
+      <c r="X357" s="274"/>
     </row>
     <row r="358" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A358" s="271" t="s">
+      <c r="A358" s="272" t="s">
         <v>242</v>
       </c>
-      <c r="B358" s="271"/>
-      <c r="C358" s="272"/>
+      <c r="B358" s="272"/>
+      <c r="C358" s="275"/>
       <c r="D358" s="174">
         <v>741298</v>
       </c>
@@ -20990,11 +20987,11 @@
       <c r="U358" s="168">
         <v>2862</v>
       </c>
-      <c r="V358" s="271" t="s">
+      <c r="V358" s="272" t="s">
         <v>242</v>
       </c>
-      <c r="W358" s="271"/>
-      <c r="X358" s="272"/>
+      <c r="W358" s="272"/>
+      <c r="X358" s="275"/>
     </row>
     <row r="359" spans="1:24" s="6" customFormat="1">
       <c r="A359" s="220"/>
@@ -21078,12 +21075,12 @@
       <c r="W361" s="93"/>
       <c r="X361" s="93"/>
     </row>
-    <row r="364" spans="1:24" s="19" customFormat="1" ht="21">
+    <row r="364" spans="1:24" s="19" customFormat="1" ht="18">
       <c r="A364" s="19" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="365" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="365" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A365" s="16"/>
       <c r="B365" s="16"/>
       <c r="C365" s="16"/>
@@ -21110,11 +21107,11 @@
       <c r="X365" s="25"/>
     </row>
     <row r="366" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A366" s="269" t="s">
+      <c r="A366" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B366" s="269"/>
-      <c r="C366" s="269"/>
+      <c r="B366" s="267"/>
+      <c r="C366" s="267"/>
       <c r="D366" s="104" t="s">
         <v>79</v>
       </c>
@@ -21169,16 +21166,16 @@
       <c r="U366" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V366" s="273" t="s">
+      <c r="V366" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W366" s="269"/>
-      <c r="X366" s="275"/>
+      <c r="W366" s="267"/>
+      <c r="X366" s="276"/>
     </row>
     <row r="367" spans="1:24" s="6" customFormat="1">
-      <c r="A367" s="270"/>
-      <c r="B367" s="270"/>
-      <c r="C367" s="270"/>
+      <c r="A367" s="268"/>
+      <c r="B367" s="268"/>
+      <c r="C367" s="268"/>
       <c r="D367" s="108" t="s">
         <v>22</v>
       </c>
@@ -21233,9 +21230,9 @@
       <c r="U367" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V367" s="274"/>
-      <c r="W367" s="270"/>
-      <c r="X367" s="276"/>
+      <c r="V367" s="270"/>
+      <c r="W367" s="268"/>
+      <c r="X367" s="277"/>
     </row>
     <row r="368" spans="1:24" s="12" customFormat="1">
       <c r="A368" s="78" t="s">
@@ -21951,7 +21948,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="381" spans="1:24" s="12" customFormat="1" ht="17.5" thickBot="1">
+    <row r="381" spans="1:24" s="12" customFormat="1" ht="15" thickBot="1">
       <c r="A381" s="84"/>
       <c r="B381" s="84"/>
       <c r="C381" s="219" t="s">
@@ -22127,7 +22124,7 @@
       <c r="W385" s="93"/>
       <c r="X385" s="93"/>
     </row>
-    <row r="388" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="388" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A388" s="19" t="s">
         <v>95</v>
       </c>
@@ -22160,11 +22157,11 @@
       <c r="X389" s="25"/>
     </row>
     <row r="390" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A390" s="269" t="s">
+      <c r="A390" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B390" s="269"/>
-      <c r="C390" s="269"/>
+      <c r="B390" s="267"/>
+      <c r="C390" s="267"/>
       <c r="D390" s="104" t="s">
         <v>79</v>
       </c>
@@ -22219,16 +22216,16 @@
       <c r="U390" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V390" s="273" t="s">
+      <c r="V390" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W390" s="269"/>
-      <c r="X390" s="275"/>
+      <c r="W390" s="267"/>
+      <c r="X390" s="276"/>
     </row>
     <row r="391" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A391" s="270"/>
-      <c r="B391" s="270"/>
-      <c r="C391" s="270"/>
+      <c r="A391" s="268"/>
+      <c r="B391" s="268"/>
+      <c r="C391" s="268"/>
       <c r="D391" s="108" t="s">
         <v>22</v>
       </c>
@@ -22283,9 +22280,9 @@
       <c r="U391" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V391" s="274"/>
-      <c r="W391" s="270"/>
-      <c r="X391" s="276"/>
+      <c r="V391" s="270"/>
+      <c r="W391" s="268"/>
+      <c r="X391" s="277"/>
     </row>
     <row r="392" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A392" s="78" t="s">
@@ -23149,7 +23146,7 @@
       <c r="W408" s="93"/>
       <c r="X408" s="93"/>
     </row>
-    <row r="411" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="411" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A411" s="19" t="s">
         <v>94</v>
       </c>
@@ -23182,11 +23179,11 @@
       <c r="X412" s="25"/>
     </row>
     <row r="413" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A413" s="269" t="s">
+      <c r="A413" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B413" s="269"/>
-      <c r="C413" s="269"/>
+      <c r="B413" s="267"/>
+      <c r="C413" s="267"/>
       <c r="D413" s="104" t="s">
         <v>79</v>
       </c>
@@ -23241,16 +23238,16 @@
       <c r="U413" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V413" s="273" t="s">
+      <c r="V413" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W413" s="269"/>
-      <c r="X413" s="275"/>
+      <c r="W413" s="267"/>
+      <c r="X413" s="276"/>
     </row>
     <row r="414" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A414" s="270"/>
-      <c r="B414" s="270"/>
-      <c r="C414" s="270"/>
+      <c r="A414" s="268"/>
+      <c r="B414" s="268"/>
+      <c r="C414" s="268"/>
       <c r="D414" s="108" t="s">
         <v>22</v>
       </c>
@@ -23305,9 +23302,9 @@
       <c r="U414" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V414" s="274"/>
-      <c r="W414" s="270"/>
-      <c r="X414" s="276"/>
+      <c r="V414" s="270"/>
+      <c r="W414" s="268"/>
+      <c r="X414" s="277"/>
     </row>
     <row r="415" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A415" s="78" t="s">
@@ -24171,7 +24168,7 @@
       <c r="W431" s="93"/>
       <c r="X431" s="93"/>
     </row>
-    <row r="434" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="434" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A434" s="19" t="s">
         <v>93</v>
       </c>
@@ -24204,11 +24201,11 @@
       <c r="X435" s="25"/>
     </row>
     <row r="436" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A436" s="269" t="s">
+      <c r="A436" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B436" s="269"/>
-      <c r="C436" s="269"/>
+      <c r="B436" s="267"/>
+      <c r="C436" s="267"/>
       <c r="D436" s="104" t="s">
         <v>79</v>
       </c>
@@ -24263,16 +24260,16 @@
       <c r="U436" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V436" s="273" t="s">
+      <c r="V436" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W436" s="269"/>
-      <c r="X436" s="275"/>
+      <c r="W436" s="267"/>
+      <c r="X436" s="276"/>
     </row>
     <row r="437" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A437" s="270"/>
-      <c r="B437" s="270"/>
-      <c r="C437" s="270"/>
+      <c r="A437" s="268"/>
+      <c r="B437" s="268"/>
+      <c r="C437" s="268"/>
       <c r="D437" s="108" t="s">
         <v>22</v>
       </c>
@@ -24327,9 +24324,9 @@
       <c r="U437" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V437" s="274"/>
-      <c r="W437" s="270"/>
-      <c r="X437" s="276"/>
+      <c r="V437" s="270"/>
+      <c r="W437" s="268"/>
+      <c r="X437" s="277"/>
     </row>
     <row r="438" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A438" s="78" t="s">
@@ -25193,13 +25190,13 @@
       <c r="W454" s="93"/>
       <c r="X454" s="93"/>
     </row>
-    <row r="457" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="457" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A457" s="19" t="s">
         <v>92</v>
       </c>
       <c r="B457" s="26"/>
     </row>
-    <row r="458" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="458" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A458" s="16"/>
       <c r="B458" s="16"/>
       <c r="C458" s="16"/>
@@ -25226,11 +25223,11 @@
       <c r="X458" s="25"/>
     </row>
     <row r="459" spans="1:24" s="6" customFormat="1" ht="33" customHeight="1">
-      <c r="A459" s="269" t="s">
+      <c r="A459" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B459" s="269"/>
-      <c r="C459" s="269"/>
+      <c r="B459" s="267"/>
+      <c r="C459" s="267"/>
       <c r="D459" s="104" t="s">
         <v>79</v>
       </c>
@@ -25285,16 +25282,16 @@
       <c r="U459" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V459" s="273" t="s">
+      <c r="V459" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W459" s="269"/>
-      <c r="X459" s="275"/>
+      <c r="W459" s="267"/>
+      <c r="X459" s="276"/>
     </row>
     <row r="460" spans="1:24" s="6" customFormat="1">
-      <c r="A460" s="270"/>
-      <c r="B460" s="270"/>
-      <c r="C460" s="270"/>
+      <c r="A460" s="268"/>
+      <c r="B460" s="268"/>
+      <c r="C460" s="268"/>
       <c r="D460" s="108" t="s">
         <v>22</v>
       </c>
@@ -25349,9 +25346,9 @@
       <c r="U460" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V460" s="274"/>
-      <c r="W460" s="270"/>
-      <c r="X460" s="276"/>
+      <c r="V460" s="270"/>
+      <c r="W460" s="268"/>
+      <c r="X460" s="277"/>
     </row>
     <row r="461" spans="1:24" s="12" customFormat="1">
       <c r="A461" s="78" t="s">
@@ -26067,7 +26064,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="474" spans="1:24" s="6" customFormat="1" ht="17.5" thickBot="1">
+    <row r="474" spans="1:24" s="6" customFormat="1" ht="15" thickBot="1">
       <c r="A474" s="84"/>
       <c r="B474" s="84"/>
       <c r="C474" s="219" t="s">
@@ -26243,7 +26240,7 @@
       <c r="W478" s="93"/>
       <c r="X478" s="93"/>
     </row>
-    <row r="481" spans="1:24" s="19" customFormat="1" ht="21">
+    <row r="481" spans="1:24" s="19" customFormat="1" ht="18">
       <c r="A481" s="19" t="s">
         <v>90</v>
       </c>
@@ -26275,11 +26272,11 @@
       <c r="X482" s="25"/>
     </row>
     <row r="483" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A483" s="269" t="s">
+      <c r="A483" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B483" s="269"/>
-      <c r="C483" s="269"/>
+      <c r="B483" s="267"/>
+      <c r="C483" s="267"/>
       <c r="D483" s="104" t="s">
         <v>79</v>
       </c>
@@ -26334,16 +26331,16 @@
       <c r="U483" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V483" s="273" t="s">
+      <c r="V483" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W483" s="269"/>
-      <c r="X483" s="275"/>
+      <c r="W483" s="267"/>
+      <c r="X483" s="276"/>
     </row>
     <row r="484" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A484" s="270"/>
-      <c r="B484" s="270"/>
-      <c r="C484" s="270"/>
+      <c r="A484" s="268"/>
+      <c r="B484" s="268"/>
+      <c r="C484" s="268"/>
       <c r="D484" s="108" t="s">
         <v>22</v>
       </c>
@@ -26398,9 +26395,9 @@
       <c r="U484" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V484" s="274"/>
-      <c r="W484" s="270"/>
-      <c r="X484" s="276"/>
+      <c r="V484" s="270"/>
+      <c r="W484" s="268"/>
+      <c r="X484" s="277"/>
     </row>
     <row r="485" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A485" s="78" t="s">
@@ -26970,7 +26967,7 @@
       <c r="W496" s="103"/>
       <c r="X496" s="103"/>
     </row>
-    <row r="499" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="499" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A499" s="19" t="s">
         <v>247</v>
       </c>
@@ -27003,11 +27000,11 @@
       <c r="X500" s="25"/>
     </row>
     <row r="501" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A501" s="269" t="s">
+      <c r="A501" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B501" s="269"/>
-      <c r="C501" s="269"/>
+      <c r="B501" s="267"/>
+      <c r="C501" s="267"/>
       <c r="D501" s="72" t="s">
         <v>79</v>
       </c>
@@ -27062,16 +27059,16 @@
       <c r="U501" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V501" s="273" t="s">
+      <c r="V501" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W501" s="269"/>
-      <c r="X501" s="269"/>
+      <c r="W501" s="267"/>
+      <c r="X501" s="267"/>
     </row>
     <row r="502" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A502" s="270"/>
-      <c r="B502" s="270"/>
-      <c r="C502" s="270"/>
+      <c r="A502" s="268"/>
+      <c r="B502" s="268"/>
+      <c r="C502" s="268"/>
       <c r="D502" s="75" t="s">
         <v>22</v>
       </c>
@@ -27126,9 +27123,9 @@
       <c r="U502" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V502" s="274"/>
-      <c r="W502" s="270"/>
-      <c r="X502" s="270"/>
+      <c r="V502" s="270"/>
+      <c r="W502" s="268"/>
+      <c r="X502" s="268"/>
     </row>
     <row r="503" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A503" s="78" t="s">
@@ -28020,7 +28017,7 @@
       <c r="W520" s="93"/>
       <c r="X520" s="93"/>
     </row>
-    <row r="523" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="523" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A523" s="19" t="s">
         <v>248</v>
       </c>
@@ -28053,11 +28050,11 @@
       <c r="X524" s="25"/>
     </row>
     <row r="525" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A525" s="269" t="s">
+      <c r="A525" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B525" s="269"/>
-      <c r="C525" s="269"/>
+      <c r="B525" s="267"/>
+      <c r="C525" s="267"/>
       <c r="D525" s="104" t="s">
         <v>79</v>
       </c>
@@ -28112,16 +28109,16 @@
       <c r="U525" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V525" s="273" t="s">
+      <c r="V525" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W525" s="269"/>
-      <c r="X525" s="269"/>
+      <c r="W525" s="267"/>
+      <c r="X525" s="267"/>
     </row>
     <row r="526" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A526" s="270"/>
-      <c r="B526" s="270"/>
-      <c r="C526" s="270"/>
+      <c r="A526" s="268"/>
+      <c r="B526" s="268"/>
+      <c r="C526" s="268"/>
       <c r="D526" s="108" t="s">
         <v>22</v>
       </c>
@@ -28176,9 +28173,9 @@
       <c r="U526" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V526" s="274"/>
-      <c r="W526" s="270"/>
-      <c r="X526" s="270"/>
+      <c r="V526" s="270"/>
+      <c r="W526" s="268"/>
+      <c r="X526" s="268"/>
     </row>
     <row r="527" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A527" s="78" t="s">
@@ -29070,7 +29067,7 @@
       <c r="W544" s="93"/>
       <c r="X544" s="93"/>
     </row>
-    <row r="547" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="547" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A547" s="19" t="s">
         <v>249</v>
       </c>
@@ -29103,11 +29100,11 @@
       <c r="X548" s="25"/>
     </row>
     <row r="549" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A549" s="269" t="s">
+      <c r="A549" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B549" s="269"/>
-      <c r="C549" s="269"/>
+      <c r="B549" s="267"/>
+      <c r="C549" s="267"/>
       <c r="D549" s="104" t="s">
         <v>79</v>
       </c>
@@ -29162,16 +29159,16 @@
       <c r="U549" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V549" s="273" t="s">
+      <c r="V549" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W549" s="269"/>
-      <c r="X549" s="269"/>
+      <c r="W549" s="267"/>
+      <c r="X549" s="267"/>
     </row>
     <row r="550" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A550" s="270"/>
-      <c r="B550" s="270"/>
-      <c r="C550" s="270"/>
+      <c r="A550" s="268"/>
+      <c r="B550" s="268"/>
+      <c r="C550" s="268"/>
       <c r="D550" s="108" t="s">
         <v>22</v>
       </c>
@@ -29226,9 +29223,9 @@
       <c r="U550" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V550" s="274"/>
-      <c r="W550" s="270"/>
-      <c r="X550" s="270"/>
+      <c r="V550" s="270"/>
+      <c r="W550" s="268"/>
+      <c r="X550" s="268"/>
     </row>
     <row r="551" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A551" s="78" t="s">
@@ -30148,7 +30145,7 @@
       <c r="W569" s="93"/>
       <c r="X569" s="93"/>
     </row>
-    <row r="572" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="572" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A572" s="19" t="s">
         <v>250</v>
       </c>
@@ -30181,11 +30178,11 @@
       <c r="X573" s="25"/>
     </row>
     <row r="574" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A574" s="269" t="s">
+      <c r="A574" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B574" s="269"/>
-      <c r="C574" s="269"/>
+      <c r="B574" s="267"/>
+      <c r="C574" s="267"/>
       <c r="D574" s="72" t="s">
         <v>79</v>
       </c>
@@ -30240,16 +30237,16 @@
       <c r="U574" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V574" s="273" t="s">
+      <c r="V574" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W574" s="269"/>
-      <c r="X574" s="269"/>
+      <c r="W574" s="267"/>
+      <c r="X574" s="267"/>
     </row>
     <row r="575" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A575" s="270"/>
-      <c r="B575" s="270"/>
-      <c r="C575" s="270"/>
+      <c r="A575" s="268"/>
+      <c r="B575" s="268"/>
+      <c r="C575" s="268"/>
       <c r="D575" s="75" t="s">
         <v>22</v>
       </c>
@@ -30304,16 +30301,16 @@
       <c r="U575" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V575" s="274"/>
-      <c r="W575" s="270"/>
-      <c r="X575" s="270"/>
+      <c r="V575" s="270"/>
+      <c r="W575" s="268"/>
+      <c r="X575" s="268"/>
     </row>
     <row r="576" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A576" s="267" t="s">
+      <c r="A576" s="278" t="s">
         <v>211</v>
       </c>
-      <c r="B576" s="267"/>
-      <c r="C576" s="268"/>
+      <c r="B576" s="278"/>
+      <c r="C576" s="279"/>
       <c r="D576" s="80">
         <v>404221.801794859</v>
       </c>
@@ -30368,18 +30365,18 @@
       <c r="U576" s="83">
         <v>0</v>
       </c>
-      <c r="V576" s="267" t="s">
+      <c r="V576" s="278" t="s">
         <v>211</v>
       </c>
-      <c r="W576" s="267"/>
-      <c r="X576" s="268"/>
+      <c r="W576" s="278"/>
+      <c r="X576" s="279"/>
     </row>
     <row r="577" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A577" s="271" t="s">
+      <c r="A577" s="272" t="s">
         <v>242</v>
       </c>
-      <c r="B577" s="271"/>
-      <c r="C577" s="272"/>
+      <c r="B577" s="272"/>
+      <c r="C577" s="275"/>
       <c r="D577" s="97">
         <v>3227127.2510000002</v>
       </c>
@@ -30434,11 +30431,11 @@
       <c r="U577" s="88">
         <v>0</v>
       </c>
-      <c r="V577" s="271" t="s">
+      <c r="V577" s="272" t="s">
         <v>242</v>
       </c>
-      <c r="W577" s="271"/>
-      <c r="X577" s="272"/>
+      <c r="W577" s="272"/>
+      <c r="X577" s="275"/>
     </row>
     <row r="578" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
       <c r="A578" s="220"/>
@@ -30550,7 +30547,7 @@
       <c r="W581" s="93"/>
       <c r="X581" s="93"/>
     </row>
-    <row r="584" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="584" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A584" s="19" t="s">
         <v>251</v>
       </c>
@@ -30583,11 +30580,11 @@
       <c r="X585" s="25"/>
     </row>
     <row r="586" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A586" s="269" t="s">
+      <c r="A586" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B586" s="269"/>
-      <c r="C586" s="269"/>
+      <c r="B586" s="267"/>
+      <c r="C586" s="267"/>
       <c r="D586" s="104" t="s">
         <v>79</v>
       </c>
@@ -30642,16 +30639,16 @@
       <c r="U586" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V586" s="273" t="s">
+      <c r="V586" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W586" s="269"/>
-      <c r="X586" s="269"/>
+      <c r="W586" s="267"/>
+      <c r="X586" s="267"/>
     </row>
     <row r="587" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A587" s="270"/>
-      <c r="B587" s="270"/>
-      <c r="C587" s="270"/>
+      <c r="A587" s="268"/>
+      <c r="B587" s="268"/>
+      <c r="C587" s="268"/>
       <c r="D587" s="108" t="s">
         <v>22</v>
       </c>
@@ -30706,9 +30703,9 @@
       <c r="U587" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V587" s="274"/>
-      <c r="W587" s="270"/>
-      <c r="X587" s="270"/>
+      <c r="V587" s="270"/>
+      <c r="W587" s="268"/>
+      <c r="X587" s="268"/>
     </row>
     <row r="588" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A588" s="79" t="s">
@@ -31602,7 +31599,7 @@
       <c r="W605" s="93"/>
       <c r="X605" s="93"/>
     </row>
-    <row r="608" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="608" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="A608" s="19" t="s">
         <v>252</v>
       </c>
@@ -31635,11 +31632,11 @@
       <c r="X609" s="25"/>
     </row>
     <row r="610" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A610" s="269" t="s">
+      <c r="A610" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="B610" s="269"/>
-      <c r="C610" s="269"/>
+      <c r="B610" s="267"/>
+      <c r="C610" s="267"/>
       <c r="D610" s="72" t="s">
         <v>79</v>
       </c>
@@ -31694,16 +31691,16 @@
       <c r="U610" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="V610" s="273" t="s">
+      <c r="V610" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="W610" s="269"/>
-      <c r="X610" s="269"/>
+      <c r="W610" s="267"/>
+      <c r="X610" s="267"/>
     </row>
     <row r="611" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A611" s="270"/>
-      <c r="B611" s="270"/>
-      <c r="C611" s="270"/>
+      <c r="A611" s="268"/>
+      <c r="B611" s="268"/>
+      <c r="C611" s="268"/>
       <c r="D611" s="75" t="s">
         <v>22</v>
       </c>
@@ -31758,9 +31755,9 @@
       <c r="U611" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="V611" s="274"/>
-      <c r="W611" s="270"/>
-      <c r="X611" s="270"/>
+      <c r="V611" s="270"/>
+      <c r="W611" s="268"/>
+      <c r="X611" s="268"/>
     </row>
     <row r="612" spans="1:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="A612" s="79" t="s">
@@ -32358,7 +32355,7 @@
       <c r="W624" s="93"/>
       <c r="X624" s="93"/>
     </row>
-    <row r="627" spans="1:24" s="6" customFormat="1" ht="21">
+    <row r="627" spans="1:24" s="6" customFormat="1" ht="18">
       <c r="B627" s="18"/>
       <c r="C627" s="24" t="s">
         <v>82</v>
@@ -32391,10 +32388,10 @@
       <c r="V628" s="15"/>
     </row>
     <row r="629" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C629" s="269" t="s">
+      <c r="C629" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D629" s="269"/>
+      <c r="D629" s="267"/>
       <c r="E629" s="104" t="s">
         <v>79</v>
       </c>
@@ -32449,14 +32446,14 @@
       <c r="V629" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W629" s="273" t="s">
+      <c r="W629" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X629" s="269"/>
+      <c r="X629" s="267"/>
     </row>
     <row r="630" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C630" s="270"/>
-      <c r="D630" s="270"/>
+      <c r="C630" s="268"/>
+      <c r="D630" s="268"/>
       <c r="E630" s="108" t="s">
         <v>22</v>
       </c>
@@ -32511,8 +32508,8 @@
       <c r="V630" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W630" s="274"/>
-      <c r="X630" s="270"/>
+      <c r="W630" s="270"/>
+      <c r="X630" s="268"/>
     </row>
     <row r="631" spans="1:24" s="6" customFormat="1" ht="15.75" customHeight="1">
       <c r="C631" s="78" t="s">
@@ -34374,7 +34371,7 @@
       <c r="W663" s="12"/>
       <c r="X663" s="12"/>
     </row>
-    <row r="666" spans="3:24" s="6" customFormat="1" ht="21">
+    <row r="666" spans="3:24" s="6" customFormat="1" ht="18">
       <c r="C666" s="19" t="s">
         <v>80</v>
       </c>
@@ -34406,10 +34403,10 @@
       <c r="X667" s="15"/>
     </row>
     <row r="668" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C668" s="269" t="s">
+      <c r="C668" s="267" t="s">
         <v>61</v>
       </c>
-      <c r="D668" s="269"/>
+      <c r="D668" s="267"/>
       <c r="E668" s="72" t="s">
         <v>79</v>
       </c>
@@ -34464,14 +34461,14 @@
       <c r="V668" s="74" t="s">
         <v>62</v>
       </c>
-      <c r="W668" s="273" t="s">
+      <c r="W668" s="269" t="s">
         <v>61</v>
       </c>
-      <c r="X668" s="269"/>
+      <c r="X668" s="267"/>
     </row>
     <row r="669" spans="3:24" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="C669" s="270"/>
-      <c r="D669" s="270"/>
+      <c r="C669" s="268"/>
+      <c r="D669" s="268"/>
       <c r="E669" s="75" t="s">
         <v>22</v>
       </c>
@@ -34526,8 +34523,8 @@
       <c r="V669" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="W669" s="274"/>
-      <c r="X669" s="270"/>
+      <c r="W669" s="270"/>
+      <c r="X669" s="268"/>
     </row>
     <row r="670" spans="3:24" s="12" customFormat="1" ht="15.75" customHeight="1">
       <c r="C670" s="78" t="s">
@@ -36409,6 +36406,59 @@
     </row>
   </sheetData>
   <mergeCells count="69">
+    <mergeCell ref="A576:C576"/>
+    <mergeCell ref="V576:X576"/>
+    <mergeCell ref="C629:D630"/>
+    <mergeCell ref="C668:D669"/>
+    <mergeCell ref="A577:C577"/>
+    <mergeCell ref="V577:X577"/>
+    <mergeCell ref="A586:C587"/>
+    <mergeCell ref="V586:X587"/>
+    <mergeCell ref="A610:C611"/>
+    <mergeCell ref="V610:X611"/>
+    <mergeCell ref="W629:X630"/>
+    <mergeCell ref="W668:X669"/>
+    <mergeCell ref="A525:C526"/>
+    <mergeCell ref="V525:X526"/>
+    <mergeCell ref="A549:C550"/>
+    <mergeCell ref="V549:X550"/>
+    <mergeCell ref="A574:C575"/>
+    <mergeCell ref="V574:X575"/>
+    <mergeCell ref="A459:C460"/>
+    <mergeCell ref="V459:X460"/>
+    <mergeCell ref="A483:C484"/>
+    <mergeCell ref="V483:X484"/>
+    <mergeCell ref="A501:C502"/>
+    <mergeCell ref="V501:X502"/>
+    <mergeCell ref="A390:C391"/>
+    <mergeCell ref="V390:X391"/>
+    <mergeCell ref="A413:C414"/>
+    <mergeCell ref="V413:X414"/>
+    <mergeCell ref="A436:C437"/>
+    <mergeCell ref="V436:X437"/>
+    <mergeCell ref="A355:C356"/>
+    <mergeCell ref="V355:X356"/>
+    <mergeCell ref="A357:C357"/>
+    <mergeCell ref="A358:C358"/>
+    <mergeCell ref="A366:C367"/>
+    <mergeCell ref="V366:X367"/>
+    <mergeCell ref="V320:X321"/>
+    <mergeCell ref="A344:C345"/>
+    <mergeCell ref="V344:X345"/>
+    <mergeCell ref="A346:C346"/>
+    <mergeCell ref="A347:C347"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="W5:X6"/>
+    <mergeCell ref="C39:D40"/>
+    <mergeCell ref="W39:X40"/>
+    <mergeCell ref="C78:D79"/>
+    <mergeCell ref="W78:X79"/>
+    <mergeCell ref="C117:D118"/>
+    <mergeCell ref="W117:X118"/>
+    <mergeCell ref="C156:D157"/>
+    <mergeCell ref="W156:X157"/>
+    <mergeCell ref="C195:D196"/>
+    <mergeCell ref="W195:X196"/>
     <mergeCell ref="C229:D230"/>
     <mergeCell ref="W229:X230"/>
     <mergeCell ref="V347:X347"/>
@@ -36425,59 +36475,6 @@
     <mergeCell ref="A312:C312"/>
     <mergeCell ref="V312:X312"/>
     <mergeCell ref="A320:C321"/>
-    <mergeCell ref="C117:D118"/>
-    <mergeCell ref="W117:X118"/>
-    <mergeCell ref="C156:D157"/>
-    <mergeCell ref="W156:X157"/>
-    <mergeCell ref="C195:D196"/>
-    <mergeCell ref="W195:X196"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="W5:X6"/>
-    <mergeCell ref="C39:D40"/>
-    <mergeCell ref="W39:X40"/>
-    <mergeCell ref="C78:D79"/>
-    <mergeCell ref="W78:X79"/>
-    <mergeCell ref="V320:X321"/>
-    <mergeCell ref="A344:C345"/>
-    <mergeCell ref="V344:X345"/>
-    <mergeCell ref="A346:C346"/>
-    <mergeCell ref="A347:C347"/>
-    <mergeCell ref="A355:C356"/>
-    <mergeCell ref="V355:X356"/>
-    <mergeCell ref="A357:C357"/>
-    <mergeCell ref="A358:C358"/>
-    <mergeCell ref="A366:C367"/>
-    <mergeCell ref="V366:X367"/>
-    <mergeCell ref="A390:C391"/>
-    <mergeCell ref="V390:X391"/>
-    <mergeCell ref="A413:C414"/>
-    <mergeCell ref="V413:X414"/>
-    <mergeCell ref="A436:C437"/>
-    <mergeCell ref="V436:X437"/>
-    <mergeCell ref="A459:C460"/>
-    <mergeCell ref="V459:X460"/>
-    <mergeCell ref="A483:C484"/>
-    <mergeCell ref="V483:X484"/>
-    <mergeCell ref="A501:C502"/>
-    <mergeCell ref="V501:X502"/>
-    <mergeCell ref="A525:C526"/>
-    <mergeCell ref="V525:X526"/>
-    <mergeCell ref="A549:C550"/>
-    <mergeCell ref="V549:X550"/>
-    <mergeCell ref="A574:C575"/>
-    <mergeCell ref="V574:X575"/>
-    <mergeCell ref="A576:C576"/>
-    <mergeCell ref="V576:X576"/>
-    <mergeCell ref="C629:D630"/>
-    <mergeCell ref="C668:D669"/>
-    <mergeCell ref="A577:C577"/>
-    <mergeCell ref="V577:X577"/>
-    <mergeCell ref="A586:C587"/>
-    <mergeCell ref="V586:X587"/>
-    <mergeCell ref="A610:C611"/>
-    <mergeCell ref="V610:X611"/>
-    <mergeCell ref="W629:X630"/>
-    <mergeCell ref="W668:X669"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -36488,23 +36485,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF1C3BCB-F422-49E0-816B-936CD0A04335}">
   <dimension ref="A1:R26"/>
-  <sheetFormatPr defaultColWidth="7.58203125" defaultRowHeight="17"/>
+  <sheetFormatPr defaultColWidth="7.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="9.83203125" customWidth="1"/>
-    <col min="3" max="3" width="9.58203125" customWidth="1"/>
-    <col min="4" max="4" width="9.75" customWidth="1"/>
-    <col min="5" max="5" width="9.5" customWidth="1"/>
-    <col min="6" max="6" width="9.08203125" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="2" max="2" width="9.77734375" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" customWidth="1"/>
+    <col min="5" max="5" width="9.44140625" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" customWidth="1"/>
     <col min="7" max="7" width="9.33203125" customWidth="1"/>
-    <col min="10" max="10" width="9.08203125" customWidth="1"/>
-    <col min="11" max="11" width="10.08203125" customWidth="1"/>
-    <col min="12" max="12" width="9.75" customWidth="1"/>
-    <col min="13" max="13" width="10.58203125" customWidth="1"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1"/>
-    <col min="15" max="15" width="9.75" customWidth="1"/>
-    <col min="16" max="16" width="10.58203125" customWidth="1"/>
-    <col min="17" max="17" width="11.08203125" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" customWidth="1"/>
+    <col min="11" max="11" width="10.109375" customWidth="1"/>
+    <col min="12" max="12" width="9.77734375" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" customWidth="1"/>
+    <col min="14" max="15" width="9.77734375" customWidth="1"/>
+    <col min="16" max="16" width="10.5546875" customWidth="1"/>
+    <col min="17" max="17" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.5" customHeight="1">
@@ -37423,13 +37419,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A557AA65-F7BB-44AB-ACFE-8282F027B7E9}">
   <dimension ref="A1:Z80"/>
-  <sheetFormatPr defaultColWidth="11.58203125" defaultRowHeight="17"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="26.58203125" customWidth="1"/>
-    <col min="2" max="2" width="11.25" customWidth="1"/>
-    <col min="3" max="3" width="11.58203125" customWidth="1"/>
-    <col min="5" max="5" width="26.58203125" customWidth="1"/>
-    <col min="9" max="26" width="17.58203125" customWidth="1"/>
+    <col min="1" max="1" width="26.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="5" max="5" width="26.5546875" customWidth="1"/>
+    <col min="9" max="26" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:8">
@@ -37711,19 +37707,19 @@
       <c r="G21" s="284"/>
       <c r="H21" s="284"/>
     </row>
-    <row r="22" spans="1:26" ht="26">
+    <row r="22" spans="1:26" ht="23.4">
       <c r="A22" s="43" t="s">
         <v>158</v>
       </c>
       <c r="L22" s="43"/>
     </row>
-    <row r="23" spans="1:26" ht="21">
+    <row r="23" spans="1:26" ht="18">
       <c r="A23" s="19" t="s">
         <v>142</v>
       </c>
       <c r="L23" s="19"/>
     </row>
-    <row r="24" spans="1:26" ht="34">
+    <row r="24" spans="1:26" ht="28.8">
       <c r="B24" s="37" t="s">
         <v>137</v>
       </c>
@@ -38044,7 +38040,7 @@
         <v>37082.316750000005</v>
       </c>
     </row>
-    <row r="28" spans="1:26">
+    <row r="28" spans="1:26" ht="15.6">
       <c r="A28" t="s">
         <v>131</v>
       </c>
@@ -38098,7 +38094,7 @@
       <c r="O33" s="53"/>
       <c r="P33" s="53"/>
     </row>
-    <row r="34" spans="1:16" ht="34">
+    <row r="34" spans="1:16" ht="28.8">
       <c r="B34" s="37" t="s">
         <v>137</v>
       </c>
@@ -38111,7 +38107,7 @@
       <c r="O34" s="53"/>
       <c r="P34" s="53"/>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" ht="15.6">
       <c r="A35" t="s">
         <v>135</v>
       </c>
@@ -38130,7 +38126,7 @@
       <c r="O35" s="53"/>
       <c r="P35" s="53"/>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" ht="15.6">
       <c r="A36" t="s">
         <v>133</v>
       </c>
@@ -38151,7 +38147,7 @@
       <c r="O36" s="53"/>
       <c r="P36" s="53"/>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" ht="15.6">
       <c r="A37" t="s">
         <v>132</v>
       </c>
@@ -38172,7 +38168,7 @@
       <c r="O37" s="53"/>
       <c r="P37" s="53"/>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" ht="15.6">
       <c r="A38" t="s">
         <v>131</v>
       </c>
@@ -38193,7 +38189,7 @@
       <c r="O38" s="53"/>
       <c r="P38" s="53"/>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:16" ht="15.6">
       <c r="E39" s="40" t="s">
         <v>138</v>
       </c>
@@ -38210,7 +38206,7 @@
       <c r="O39" s="53"/>
       <c r="P39" s="53"/>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" ht="15.6">
       <c r="E40" s="40" t="s">
         <v>207</v>
       </c>
@@ -38227,7 +38223,7 @@
       <c r="O40" s="53"/>
       <c r="P40" s="53"/>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" ht="15.6">
       <c r="E41" s="39"/>
       <c r="L41" s="2"/>
       <c r="M41" s="55"/>
@@ -38235,12 +38231,12 @@
       <c r="O41" s="53"/>
       <c r="P41" s="53"/>
     </row>
-    <row r="42" spans="1:16" ht="21">
+    <row r="42" spans="1:16" ht="18">
       <c r="A42" s="19" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="34">
+    <row r="43" spans="1:16" ht="28.8">
       <c r="B43" s="37" t="s">
         <v>137</v>
       </c>
@@ -38355,7 +38351,7 @@
       <c r="S58" s="32"/>
       <c r="T58" s="32"/>
     </row>
-    <row r="59" spans="1:20" ht="21">
+    <row r="59" spans="1:20" ht="18">
       <c r="A59" s="61"/>
       <c r="L59" s="2"/>
       <c r="M59" s="41"/>
@@ -38388,7 +38384,7 @@
       <c r="F65" s="49"/>
       <c r="G65" s="49"/>
     </row>
-    <row r="66" spans="1:7" ht="21">
+    <row r="66" spans="1:7" ht="18">
       <c r="A66" s="61"/>
     </row>
     <row r="67" spans="1:7">
@@ -38410,7 +38406,7 @@
       <c r="B71" s="53"/>
       <c r="F71" s="53"/>
     </row>
-    <row r="73" spans="1:7" ht="21">
+    <row r="73" spans="1:7" ht="18">
       <c r="A73" s="61"/>
       <c r="B73" s="38"/>
     </row>
@@ -38456,7 +38452,7 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultRowHeight="17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="4" width="23.33203125" customWidth="1"/>
   </cols>
@@ -38479,15 +38475,15 @@
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="46">
+      <c r="B2" s="41">
         <f>Calculations!F4</f>
         <v>0</v>
       </c>
-      <c r="C2" s="46">
+      <c r="C2" s="41">
         <f>Calculations!G4</f>
         <v>0</v>
       </c>
-      <c r="D2" s="46">
+      <c r="D2" s="41">
         <f>Calculations!H4</f>
         <v>0</v>
       </c>
@@ -38496,15 +38492,15 @@
       <c r="A3" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="B3" s="46">
+      <c r="B3" s="41">
         <f>Calculations!F5</f>
         <v>0</v>
       </c>
-      <c r="C3" s="46">
+      <c r="C3" s="41">
         <f>Calculations!G5</f>
         <v>0</v>
       </c>
-      <c r="D3" s="46">
+      <c r="D3" s="41">
         <f>Calculations!H5</f>
         <v>0</v>
       </c>
@@ -38513,13 +38509,13 @@
       <c r="A4" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="B4" s="46">
-        <v>0</v>
-      </c>
-      <c r="C4" s="46">
-        <v>0</v>
-      </c>
-      <c r="D4" s="46">
+      <c r="B4" s="41">
+        <v>0</v>
+      </c>
+      <c r="C4" s="41">
+        <v>0</v>
+      </c>
+      <c r="D4" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38527,15 +38523,15 @@
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="46">
+      <c r="B5" s="41">
         <f>Calculations!F6</f>
         <v>0</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="41">
         <f>Calculations!G6</f>
         <v>0</v>
       </c>
-      <c r="D5" s="46">
+      <c r="D5" s="41">
         <f>Calculations!H6</f>
         <v>0</v>
       </c>
@@ -38544,15 +38540,15 @@
       <c r="A6" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="46">
+      <c r="B6" s="41">
         <f>Calculations!F7</f>
         <v>0</v>
       </c>
-      <c r="C6" s="46">
+      <c r="C6" s="41">
         <f>Calculations!G7</f>
         <v>0.09</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="41">
         <f>Calculations!H7</f>
         <v>1.079</v>
       </c>
@@ -38561,15 +38557,15 @@
       <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="41">
         <f>Calculations!F8</f>
         <v>0</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="41">
         <f>Calculations!G8</f>
         <v>8.60351</v>
       </c>
-      <c r="D7" s="46">
+      <c r="D7" s="41">
         <f>Calculations!H8</f>
         <v>5.0520199999999997</v>
       </c>
@@ -38578,15 +38574,15 @@
       <c r="A8" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="41">
         <f>Calculations!F9</f>
         <v>2153.5204869029099</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="41">
         <f>Calculations!G9</f>
         <v>358.12386349709004</v>
       </c>
-      <c r="D8" s="289">
+      <c r="D8" s="41">
         <f>Calculations!H9</f>
         <v>1335.48326537</v>
       </c>
@@ -38595,15 +38591,15 @@
       <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="46">
+      <c r="B9" s="41">
         <f>Calculations!F10</f>
         <v>0</v>
       </c>
-      <c r="C9" s="46">
+      <c r="C9" s="41">
         <f>Calculations!G10</f>
         <v>0</v>
       </c>
-      <c r="D9" s="46">
+      <c r="D9" s="41">
         <f>Calculations!H10</f>
         <v>0</v>
       </c>
@@ -38612,15 +38608,15 @@
       <c r="A10" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="41">
         <f>Calculations!F11</f>
         <v>0</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="41">
         <f>Calculations!G11</f>
         <v>0</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="41">
         <f>Calculations!H11</f>
         <v>0</v>
       </c>
@@ -38629,15 +38625,15 @@
       <c r="A11" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="46">
+      <c r="B11" s="41">
         <f>Calculations!F12</f>
         <v>0</v>
       </c>
-      <c r="C11" s="46">
+      <c r="C11" s="41">
         <f>Calculations!G12</f>
         <v>0</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="41">
         <f>Calculations!H12</f>
         <v>0</v>
       </c>
@@ -38646,15 +38642,15 @@
       <c r="A12" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="41">
         <f>Calculations!F13</f>
         <v>0</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="41">
         <f>Calculations!G13</f>
         <v>0</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="41">
         <f>Calculations!H13</f>
         <v>0</v>
       </c>
@@ -38663,15 +38659,15 @@
       <c r="A13" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="46">
+      <c r="B13" s="41">
         <f>Calculations!F14</f>
         <v>0</v>
       </c>
-      <c r="C13" s="46">
+      <c r="C13" s="41">
         <f>Calculations!G14</f>
         <v>0</v>
       </c>
-      <c r="D13" s="46">
+      <c r="D13" s="41">
         <f>Calculations!H14</f>
         <v>0</v>
       </c>
@@ -38680,15 +38676,15 @@
       <c r="A14" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="46">
+      <c r="B14" s="41">
         <f>Calculations!F15</f>
         <v>0</v>
       </c>
-      <c r="C14" s="46">
+      <c r="C14" s="41">
         <f>Calculations!G15</f>
         <v>0</v>
       </c>
-      <c r="D14" s="46">
+      <c r="D14" s="41">
         <f>Calculations!H15</f>
         <v>0</v>
       </c>
@@ -38697,15 +38693,15 @@
       <c r="A15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="46">
+      <c r="B15" s="41">
         <f>Calculations!F16</f>
         <v>0</v>
       </c>
-      <c r="C15" s="46">
+      <c r="C15" s="41">
         <f>Calculations!G16</f>
         <v>0</v>
       </c>
-      <c r="D15" s="46">
+      <c r="D15" s="41">
         <f>Calculations!H16</f>
         <v>0</v>
       </c>
@@ -38714,15 +38710,15 @@
       <c r="A16" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="46">
+      <c r="B16" s="41">
         <f>Calculations!F17</f>
         <v>0</v>
       </c>
-      <c r="C16" s="46">
+      <c r="C16" s="41">
         <f>Calculations!G17</f>
         <v>0</v>
       </c>
-      <c r="D16" s="46">
+      <c r="D16" s="41">
         <f>Calculations!H17</f>
         <v>0</v>
       </c>
@@ -38731,15 +38727,15 @@
       <c r="A17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="46">
+      <c r="B17" s="41">
         <f>Calculations!F18</f>
         <v>0</v>
       </c>
-      <c r="C17" s="46">
+      <c r="C17" s="41">
         <f>Calculations!G18</f>
         <v>0</v>
       </c>
-      <c r="D17" s="46">
+      <c r="D17" s="41">
         <f>Calculations!H18</f>
         <v>0</v>
       </c>
@@ -38748,15 +38744,15 @@
       <c r="A18" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="46">
+      <c r="B18" s="41">
         <f>Calculations!F19</f>
         <v>0</v>
       </c>
-      <c r="C18" s="46">
+      <c r="C18" s="41">
         <f>Calculations!G19</f>
         <v>0</v>
       </c>
-      <c r="D18" s="46">
+      <c r="D18" s="41">
         <f>Calculations!H19</f>
         <v>0</v>
       </c>
@@ -38765,13 +38761,13 @@
       <c r="A19" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="B19" s="46">
-        <v>0</v>
-      </c>
-      <c r="C19" s="46">
-        <v>0</v>
-      </c>
-      <c r="D19" s="46">
+      <c r="B19" s="41">
+        <v>0</v>
+      </c>
+      <c r="C19" s="41">
+        <v>0</v>
+      </c>
+      <c r="D19" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38779,13 +38775,13 @@
       <c r="A20" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="B20" s="46">
-        <v>0</v>
-      </c>
-      <c r="C20" s="46">
-        <v>0</v>
-      </c>
-      <c r="D20" s="46">
+      <c r="B20" s="41">
+        <v>0</v>
+      </c>
+      <c r="C20" s="41">
+        <v>0</v>
+      </c>
+      <c r="D20" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38793,13 +38789,13 @@
       <c r="A21" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="B21" s="46">
-        <v>0</v>
-      </c>
-      <c r="C21" s="46">
-        <v>0</v>
-      </c>
-      <c r="D21" s="46">
+      <c r="B21" s="41">
+        <v>0</v>
+      </c>
+      <c r="C21" s="41">
+        <v>0</v>
+      </c>
+      <c r="D21" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38807,13 +38803,13 @@
       <c r="A22" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="B22" s="46">
-        <v>0</v>
-      </c>
-      <c r="C22" s="46">
-        <v>0</v>
-      </c>
-      <c r="D22" s="46">
+      <c r="B22" s="41">
+        <v>0</v>
+      </c>
+      <c r="C22" s="41">
+        <v>0</v>
+      </c>
+      <c r="D22" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38821,13 +38817,13 @@
       <c r="A23" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="B23" s="46">
-        <v>0</v>
-      </c>
-      <c r="C23" s="46">
-        <v>0</v>
-      </c>
-      <c r="D23" s="46">
+      <c r="B23" s="41">
+        <v>0</v>
+      </c>
+      <c r="C23" s="41">
+        <v>0</v>
+      </c>
+      <c r="D23" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38835,13 +38831,13 @@
       <c r="A24" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="B24" s="46">
-        <v>0</v>
-      </c>
-      <c r="C24" s="46">
-        <v>0</v>
-      </c>
-      <c r="D24" s="46">
+      <c r="B24" s="41">
+        <v>0</v>
+      </c>
+      <c r="C24" s="41">
+        <v>0</v>
+      </c>
+      <c r="D24" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38849,13 +38845,13 @@
       <c r="A25" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B25" s="46">
-        <v>0</v>
-      </c>
-      <c r="C25" s="46">
-        <v>0</v>
-      </c>
-      <c r="D25" s="46">
+      <c r="B25" s="41">
+        <v>0</v>
+      </c>
+      <c r="C25" s="41">
+        <v>0</v>
+      </c>
+      <c r="D25" s="41">
         <v>0</v>
       </c>
     </row>
@@ -38867,6 +38863,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -39010,15 +39015,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -39026,13 +39022,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5081983-C054-4D21-B9DE-295F402E9DEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C13E5099-7325-43F2-B9AF-DDA913304CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C13E5099-7325-43F2-B9AF-DDA913304CE9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5081983-C054-4D21-B9DE-295F402E9DEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E0DFE3B-646D-4DF2-B7F0-FAF7606D292A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E0DFE3B-646D-4DF2-B7F0-FAF7606D292A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>